<commit_message>
Fill #13 Pix2Graph real metrics (n=200) into Implement r21
#13 full run (P100 fp16, inference-only): graph-aug VQA. Acc=0.485,
Prec=0.4463, Recall=0.448, F1=0.4327; baseline no-graph 0.460 (gain +0.025).
Infer 1575s, Steps=0. Also: _build.py 14 slug fix, #13 full notebook.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JOUR-2026.xlsx
+++ b/JOUR-2026.xlsx
@@ -3526,22 +3526,70 @@
           <t xml:space="preserve">      Pix2Graph</t>
         </is>
       </c>
-      <c r="D21" s="84" t="n"/>
-      <c r="E21" s="84" t="n"/>
-      <c r="F21" s="84" t="n"/>
-      <c r="G21" s="84" t="n"/>
-      <c r="H21" s="84" t="n"/>
-      <c r="I21" s="84" t="n"/>
-      <c r="J21" s="84" t="n"/>
-      <c r="K21" s="84" t="n"/>
-      <c r="L21" s="84" t="n"/>
-      <c r="M21" s="84" t="n"/>
-      <c r="N21" s="84" t="n"/>
-      <c r="O21" s="84" t="n"/>
-      <c r="P21" s="84" t="n"/>
-      <c r="Q21" s="84" t="n"/>
-      <c r="R21" s="91" t="n"/>
-      <c r="S21" s="24" t="n"/>
+      <c r="D21" s="84" t="inlineStr">
+        <is>
+          <t>Open-vocab Scene Graph Gen -&gt; adapt sang graph-augmented VQA</t>
+        </is>
+      </c>
+      <c r="E21" s="84" t="inlineStr">
+        <is>
+          <t>Image-&gt;scene-graph sequence (PGSG-style prompt) -&gt; parse triplets -&gt; inject as VQA context</t>
+        </is>
+      </c>
+      <c r="F21" s="84" t="inlineStr">
+        <is>
+          <t>Inference-only (khong train); Qwen2.5-VL-3B sinh graph + tra loi VQA</t>
+        </is>
+      </c>
+      <c r="G21" s="84" t="n">
+        <v>0.485</v>
+      </c>
+      <c r="H21" s="84" t="n">
+        <v>0.4463</v>
+      </c>
+      <c r="I21" s="84" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="J21" s="84" t="n">
+        <v>0.4327</v>
+      </c>
+      <c r="K21" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L21" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M21" s="84" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="N21" s="84" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="O21" s="84" t="n">
+        <v>1575.4</v>
+      </c>
+      <c r="P21" s="84" t="inlineStr">
+        <is>
+          <t>~3B; inference-only (fp16, P100 sm_60)</t>
+        </is>
+      </c>
+      <c r="Q21" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R21" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="24" t="inlineStr">
+        <is>
+          <t>Qwen2.5-VL-3B; Visual CoT-GQA; eval=200; inference-only (Steps=0). ADAPTATION (Nhanh A): PGSG goc la SGG (Recall@K) -&gt; adapt sang graph-augmented VQA: Qwen sinh scene graph 2 seq (nucleus p=0.9, T=0.7) -&gt; parse triplet 's-p-o' (Qwen khong co token [ENT]/[REL] cua paper -&gt; dung text + regex) -&gt; inject vao prompt VQA. Graph-aug Acc=0.4850; baseline no-graph Acc=0.4600 (gain +0.0250). ROC/PR-AUC=N/A (khong rerank); Recall@K=N/A (Visual CoT-GQA khong co gold scene graph). adaptation, not full PGSG reproduction (paper: BLIP SGG, PSG/VG/OIv6, R@K).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="132" t="n"/>

</xml_diff>

<commit_message>
Fill #14 MR-MKG real metrics (n=200) into Implement r20
#14 full run (P100 fp16, inference-only, CLIP-cosine retrieval): Acc=0.46,
Prec=0.4227, Recall=0.4112, F1=0.4005. baseline no-knowledge 0.46 (gain 0
at n=200). Infer 1945s, Steps=0.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JOUR-2026.xlsx
+++ b/JOUR-2026.xlsx
@@ -3485,34 +3485,66 @@
       </c>
       <c r="D20" s="84" t="inlineStr">
         <is>
-          <t>Multimodal VQA + structured 4-stage CoT reasoning</t>
+          <t>Multimodal reasoning + MMKG -&gt; adapt sang knowledge-injected VQA</t>
         </is>
       </c>
       <c r="E20" s="84" t="inlineStr">
         <is>
-          <t>QLoRA SFT 4-stage (SUMMARY/CAPTION/REASONING/CONCLUSION); optional SWIRES</t>
+          <t>Build MMKG (VLM scene graph) -&gt; retrieve Top-N question-relevant triples -&gt; inject as knowledge context -&gt; VQA</t>
         </is>
       </c>
       <c r="F20" s="84" t="inlineStr">
         <is>
-          <t>QLoRA r=8 on Qwen2.5-VL-3B (vision encoder frozen)</t>
-        </is>
-      </c>
-      <c r="G20" s="84" t="n"/>
-      <c r="H20" s="84" t="n"/>
-      <c r="I20" s="84" t="n"/>
-      <c r="J20" s="84" t="n"/>
-      <c r="K20" s="84" t="n"/>
-      <c r="L20" s="84" t="n"/>
-      <c r="M20" s="84" t="n"/>
-      <c r="N20" s="84" t="n"/>
-      <c r="O20" s="87" t="n"/>
-      <c r="P20" s="84" t="n"/>
-      <c r="Q20" s="84" t="n"/>
-      <c r="R20" s="84" t="n"/>
+          <t>Inference-only (khong train); Qwen2.5-VL-3B lam VLM + MMKG builder</t>
+        </is>
+      </c>
+      <c r="G20" s="84" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H20" s="84" t="n">
+        <v>0.4227</v>
+      </c>
+      <c r="I20" s="84" t="n">
+        <v>0.4112</v>
+      </c>
+      <c r="J20" s="84" t="n">
+        <v>0.4005</v>
+      </c>
+      <c r="K20" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L20" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M20" s="84" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="N20" s="84" t="n">
+        <v>0.5888</v>
+      </c>
+      <c r="O20" s="87" t="n">
+        <v>1945.4</v>
+      </c>
+      <c r="P20" s="84" t="inlineStr">
+        <is>
+          <t>~3B; inference-only (fp16, P100 sm_60)</t>
+        </is>
+      </c>
+      <c r="Q20" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R20" s="84" t="n">
+        <v>0</v>
+      </c>
       <c r="S20" s="88" t="inlineStr">
         <is>
-          <t>LLaVA-CoT full run v11 (P100, fp16, 32 steps): training COLLAPSED — model emits degenerate output (Acc=0.0). Likely fp16 instability / vision-encoder overflow on sm_60 (no bf16). Re-running with stability fix (LR 2e-4-&gt;1e-4, max_grad_norm 0.5, warmup_ratio 0.1). Metrics pending.</t>
+          <t>Qwen2.5-VL-3B; Visual CoT-GQA; eval=200; inference-only (Steps=0). ADAPTATION: MR-MKG goc = RGAT tren MMKG + knowledge adapter + cross-modal align + QLoRA (LLM+visual frozen, train ~2.25%), dung scene graph VG, ScienceQA/MARS. -&gt; Adapt: build MMKG tu scene graph do VLM sinh (2 seq, p=0.9) -&gt; retrieve Top-5 triple bang CLIP cosine + 1-hop (paper §A.6; giong sub-MMKG retrieval) -&gt; inject nhu knowledge context (RGAT+adapter -&gt; prompt, do KHONG co sceneGraphs.json va RGAT nang) -&gt; VQA. KHONG dung truong reasoning/thought (gold-leaking). Knowledge-inj Acc=0.4600; baseline Acc=0.4600 (gain +0.0000). Hits@1/ROC/PR-AUC=N/A (EM VQA). Faithful RGAT+triplet+QLoRA = future work (can GQA sceneGraphs.json). adaptation, not full MR-MKG reproduction.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix sheet: #14 MR-MKG was in r20 (STT12 row) -> move to r22; restore r20 (LLaVA-CoT)
Data-integrity fix: I had filled #14 MR-MKG metrics into row 20, but row 20
is STT 12 (LLaVA-CoT). Moved #14 to its correct row 22; restored r20 to
LLaVA-CoT (descriptive cols + updated collapse/generation-bug note, metrics blank).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JOUR-2026.xlsx
+++ b/JOUR-2026.xlsx
@@ -3485,66 +3485,34 @@
       </c>
       <c r="D20" s="84" t="inlineStr">
         <is>
-          <t>Multimodal reasoning + MMKG -&gt; adapt sang knowledge-injected VQA</t>
+          <t>Multimodal VQA + structured 4-stage CoT reasoning</t>
         </is>
       </c>
       <c r="E20" s="84" t="inlineStr">
         <is>
-          <t>Build MMKG (VLM scene graph) -&gt; retrieve Top-N question-relevant triples -&gt; inject as knowledge context -&gt; VQA</t>
+          <t>QLoRA SFT 4-stage (SUMMARY/CAPTION/REASONING/CONCLUSION); optional SWIRES</t>
         </is>
       </c>
       <c r="F20" s="84" t="inlineStr">
         <is>
-          <t>Inference-only (khong train); Qwen2.5-VL-3B lam VLM + MMKG builder</t>
-        </is>
-      </c>
-      <c r="G20" s="84" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="H20" s="84" t="n">
-        <v>0.4227</v>
-      </c>
-      <c r="I20" s="84" t="n">
-        <v>0.4112</v>
-      </c>
-      <c r="J20" s="84" t="n">
-        <v>0.4005</v>
-      </c>
-      <c r="K20" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L20" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M20" s="84" t="n">
-        <v>0.0014</v>
-      </c>
-      <c r="N20" s="84" t="n">
-        <v>0.5888</v>
-      </c>
-      <c r="O20" s="87" t="n">
-        <v>1945.4</v>
-      </c>
-      <c r="P20" s="84" t="inlineStr">
-        <is>
-          <t>~3B; inference-only (fp16, P100 sm_60)</t>
-        </is>
-      </c>
-      <c r="Q20" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R20" s="84" t="n">
-        <v>0</v>
-      </c>
+          <t>QLoRA r=8 on Qwen2.5-VL-3B (vision encoder frozen)</t>
+        </is>
+      </c>
+      <c r="G20" s="84" t="n"/>
+      <c r="H20" s="84" t="n"/>
+      <c r="I20" s="84" t="n"/>
+      <c r="J20" s="84" t="n"/>
+      <c r="K20" s="84" t="n"/>
+      <c r="L20" s="84" t="n"/>
+      <c r="M20" s="84" t="n"/>
+      <c r="N20" s="84" t="n"/>
+      <c r="O20" s="87" t="n"/>
+      <c r="P20" s="84" t="n"/>
+      <c r="Q20" s="84" t="n"/>
+      <c r="R20" s="84" t="n"/>
       <c r="S20" s="88" t="inlineStr">
         <is>
-          <t>Qwen2.5-VL-3B; Visual CoT-GQA; eval=200; inference-only (Steps=0). ADAPTATION: MR-MKG goc = RGAT tren MMKG + knowledge adapter + cross-modal align + QLoRA (LLM+visual frozen, train ~2.25%), dung scene graph VG, ScienceQA/MARS. -&gt; Adapt: build MMKG tu scene graph do VLM sinh (2 seq, p=0.9) -&gt; retrieve Top-5 triple bang CLIP cosine + 1-hop (paper §A.6; giong sub-MMKG retrieval) -&gt; inject nhu knowledge context (RGAT+adapter -&gt; prompt, do KHONG co sceneGraphs.json va RGAT nang) -&gt; VQA. KHONG dung truong reasoning/thought (gold-leaking). Knowledge-inj Acc=0.4600; baseline Acc=0.4600 (gain +0.0000). Hits@1/ROC/PR-AUC=N/A (EM VQA). Faithful RGAT+triplet+QLoRA = future work (can GQA sceneGraphs.json). adaptation, not full MR-MKG reproduction.</t>
+          <t>LLaVA-CoT (Qwen2.5-VL-3B QLoRA r=8, Visual CoT-GQA, train=256/32 steps). Training STABLE after fix (loss 1.39-&gt;0.58; LR 1e-4, grad-clip 0.5, warmup, MAX_PIXELS 200704) nhung GENERATION bi garbage (model xuat '\[\[' lap, Acc=0.0) -&gt; loi generation rieng (khong phai divergence). Metrics pending fix generation (repetition_penalty / giam max_new / tang steps).</t>
         </is>
       </c>
     </row>
@@ -3633,22 +3601,70 @@
           <t xml:space="preserve">       MR-MKG</t>
         </is>
       </c>
-      <c r="D22" s="84" t="n"/>
-      <c r="E22" s="84" t="n"/>
-      <c r="F22" s="84" t="n"/>
-      <c r="G22" s="84" t="n"/>
-      <c r="H22" s="84" t="n"/>
-      <c r="I22" s="84" t="n"/>
-      <c r="J22" s="84" t="n"/>
-      <c r="K22" s="84" t="n"/>
-      <c r="L22" s="84" t="n"/>
-      <c r="M22" s="84" t="n"/>
-      <c r="N22" s="84" t="n"/>
-      <c r="O22" s="84" t="n"/>
-      <c r="P22" s="84" t="n"/>
-      <c r="Q22" s="84" t="n"/>
-      <c r="R22" s="84" t="n"/>
-      <c r="S22" s="24" t="n"/>
+      <c r="D22" s="84" t="inlineStr">
+        <is>
+          <t>Multimodal reasoning + MMKG -&gt; adapt sang knowledge-injected VQA</t>
+        </is>
+      </c>
+      <c r="E22" s="84" t="inlineStr">
+        <is>
+          <t>Build MMKG (VLM scene graph) -&gt; retrieve Top-N question-relevant triples -&gt; inject as knowledge context -&gt; VQA</t>
+        </is>
+      </c>
+      <c r="F22" s="84" t="inlineStr">
+        <is>
+          <t>Inference-only (khong train); Qwen2.5-VL-3B lam VLM + MMKG builder</t>
+        </is>
+      </c>
+      <c r="G22" s="84" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="H22" s="84" t="n">
+        <v>0.4227</v>
+      </c>
+      <c r="I22" s="84" t="n">
+        <v>0.4112</v>
+      </c>
+      <c r="J22" s="84" t="n">
+        <v>0.4005</v>
+      </c>
+      <c r="K22" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L22" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M22" s="84" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="N22" s="84" t="n">
+        <v>0.5888</v>
+      </c>
+      <c r="O22" s="84" t="n">
+        <v>1945.4</v>
+      </c>
+      <c r="P22" s="84" t="inlineStr">
+        <is>
+          <t>~3B; inference-only (fp16, P100 sm_60)</t>
+        </is>
+      </c>
+      <c r="Q22" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R22" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="24" t="inlineStr">
+        <is>
+          <t>Qwen2.5-VL-3B; Visual CoT-GQA; eval=200; inference-only (Steps=0). ADAPTATION: MR-MKG goc = RGAT tren MMKG + knowledge adapter + cross-modal align + QLoRA (LLM+visual frozen, train ~2.25%), dung scene graph VG, ScienceQA/MARS. -&gt; Adapt: build MMKG tu scene graph do VLM sinh (2 seq, p=0.9) -&gt; retrieve Top-5 triple bang CLIP cosine + 1-hop (paper §A.6; giong sub-MMKG retrieval) -&gt; inject nhu knowledge context (RGAT+adapter -&gt; prompt, do KHONG co sceneGraphs.json va RGAT nang) -&gt; VQA. KHONG dung truong reasoning/thought (gold-leaking). Knowledge-inj Acc=0.4600; baseline Acc=0.4600 (gain +0.0000). Hits@1/ROC/PR-AUC=N/A (EM VQA). Faithful RGAT+triplet+QLoRA = future work (can GQA sceneGraphs.json). adaptation, not full MR-MKG reproduction.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="133" t="n"/>

</xml_diff>

<commit_message>
#12 LLaVA-CoT: fix gen-collapse + two-stage extraction; fill r20 (n=200)
- Generation collapse after QLoRA (greedy -> degenerate tokens): switch to
  sampling + repetition_penalty=1.15, temp=0.3, max_new=256, eval prompt
  matching the trained <CONCLUSION> format.
- Acc=0.0 from verbose CONCLUSION (Qwen2.5-VL-3B emits full sentences where
  GQA wants 1-2 words): two-stage extraction -- use <CONCLUSION> when short
  (<=6 words), else short_answer() greedy 1-5 words conditioned on the CoT.
- Full run v15 (train=256, eval=200): Acc 0.51, P/R/F1 0.4829/0.4675/0.4606,
  FPR/FNR 0.0015/0.5325, TrainTime 684.4s, Steps 64. Filled into Implement r20.
- Rebuild #12 notebooks; carry #11/#14 notebook rebuild drift + #11 summary.
- _build.py: drop leftover #15 config (#15 out of scope).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JOUR-2026.xlsx
+++ b/JOUR-2026.xlsx
@@ -3498,21 +3498,53 @@
           <t>QLoRA r=8 on Qwen2.5-VL-3B (vision encoder frozen)</t>
         </is>
       </c>
-      <c r="G20" s="84" t="n"/>
-      <c r="H20" s="84" t="n"/>
-      <c r="I20" s="84" t="n"/>
-      <c r="J20" s="84" t="n"/>
-      <c r="K20" s="84" t="n"/>
-      <c r="L20" s="84" t="n"/>
-      <c r="M20" s="84" t="n"/>
-      <c r="N20" s="84" t="n"/>
-      <c r="O20" s="87" t="n"/>
-      <c r="P20" s="84" t="n"/>
-      <c r="Q20" s="84" t="n"/>
-      <c r="R20" s="84" t="n"/>
+      <c r="G20" s="84" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H20" s="84" t="n">
+        <v>0.4829</v>
+      </c>
+      <c r="I20" s="84" t="n">
+        <v>0.4675</v>
+      </c>
+      <c r="J20" s="84" t="n">
+        <v>0.4606</v>
+      </c>
+      <c r="K20" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L20" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M20" s="84" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="N20" s="84" t="n">
+        <v>0.5325</v>
+      </c>
+      <c r="O20" s="87" t="n">
+        <v>684.4</v>
+      </c>
+      <c r="P20" s="84" t="inlineStr">
+        <is>
+          <t>~3B; LoRA 18576384</t>
+        </is>
+      </c>
+      <c r="Q20" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R20" s="84" t="n">
+        <v>64</v>
+      </c>
       <c r="S20" s="88" t="inlineStr">
         <is>
-          <t>LLaVA-CoT (Qwen2.5-VL-3B QLoRA r=8, Visual CoT-GQA, train=256/32 steps). Training STABLE after fix (loss 1.39-&gt;0.58; LR 1e-4, grad-clip 0.5, warmup, MAX_PIXELS 200704) nhung GENERATION bi garbage (model xuat '\[\[' lap, Acc=0.0) -&gt; loi generation rieng (khong phai divergence). Metrics pending fix generation (repetition_penalty / giam max_new / tang steps).</t>
+          <t>Qwen2.5-VL-3B; Visual CoT-GQA; train=256; eval=200; 4-stage structured CoT SFT (QLoRA r=8); Acc=EM, macro P/R/F1 over gold classes; answer = &lt;CONCLUSION&gt; content neu ngan (&lt;=6 words), nguoc lai stage-2 short-answer re-gen (Qwen thien verbose; paper Sec 3.1.1 conclusion ngan/dai tuy y); adaptation, not full LLaVA-CoT reproduction (paper: Llama-3.2-11B full FT). Appendix C/D (lr, SWIRES M/N/C/threshold) not in this paper version.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JOUR-2026 sheet: uniform number format for Phuc rows (19-23); strip paper-name ws
Phuc metric cells were 'General'-formatted so decimals showed inconsistently
(0.4 vs 0.4216 vs 0.51). Apply 0.0000 (Acc/Prec/Recall/F1/ROC/PR/FPR/FNR),
#,##0.0 (Train Time), 0 (Steps). Values were already correct floats -- display
only. Also strip leading whitespace in Paper names (Pix2Graph, MR-MKG).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JOUR-2026.xlsx
+++ b/JOUR-2026.xlsx
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy.m"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="41">
     <font>
@@ -437,7 +439,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -810,6 +812,21 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="167" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="167" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3427,31 +3444,31 @@
           <t>Inference-only (khong train); Qwen2.5-VL-3B 4-bit lam VLM + reasoner</t>
         </is>
       </c>
-      <c r="G19" s="84" t="n">
+      <c r="G19" s="137" t="n">
         <v>0.4</v>
       </c>
-      <c r="H19" s="84" t="n">
+      <c r="H19" s="137" t="n">
         <v>0.4216</v>
       </c>
-      <c r="I19" s="84" t="n">
+      <c r="I19" s="137" t="n">
         <v>0.3792</v>
       </c>
-      <c r="J19" s="84" t="n">
+      <c r="J19" s="137" t="n">
         <v>0.382</v>
       </c>
-      <c r="K19" s="84" t="n">
+      <c r="K19" s="137" t="n">
         <v>0.539</v>
       </c>
-      <c r="L19" s="84" t="n">
+      <c r="L19" s="137" t="n">
         <v>0.5016</v>
       </c>
-      <c r="M19" s="84" t="n">
+      <c r="M19" s="137" t="n">
         <v>0.001</v>
       </c>
-      <c r="N19" s="84" t="n">
+      <c r="N19" s="137" t="n">
         <v>0.6208</v>
       </c>
-      <c r="O19" s="84" t="n">
+      <c r="O19" s="138" t="n">
         <v>7654.5</v>
       </c>
       <c r="P19" s="84" t="inlineStr">
@@ -3464,7 +3481,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R19" s="84" t="n">
+      <c r="R19" s="139" t="n">
         <v>0</v>
       </c>
       <c r="S19" s="24" t="inlineStr">
@@ -3498,35 +3515,35 @@
           <t>QLoRA r=8 on Qwen2.5-VL-3B (vision encoder frozen)</t>
         </is>
       </c>
-      <c r="G20" s="84" t="n">
+      <c r="G20" s="137" t="n">
         <v>0.51</v>
       </c>
-      <c r="H20" s="84" t="n">
+      <c r="H20" s="137" t="n">
         <v>0.4829</v>
       </c>
-      <c r="I20" s="84" t="n">
+      <c r="I20" s="137" t="n">
         <v>0.4675</v>
       </c>
-      <c r="J20" s="84" t="n">
+      <c r="J20" s="137" t="n">
         <v>0.4606</v>
       </c>
-      <c r="K20" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L20" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M20" s="84" t="n">
+      <c r="K20" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L20" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M20" s="137" t="n">
         <v>0.0015</v>
       </c>
-      <c r="N20" s="84" t="n">
+      <c r="N20" s="137" t="n">
         <v>0.5325</v>
       </c>
-      <c r="O20" s="87" t="n">
+      <c r="O20" s="140" t="n">
         <v>684.4</v>
       </c>
       <c r="P20" s="84" t="inlineStr">
@@ -3539,7 +3556,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R20" s="84" t="n">
+      <c r="R20" s="139" t="n">
         <v>64</v>
       </c>
       <c r="S20" s="88" t="inlineStr">
@@ -3555,7 +3572,7 @@
       </c>
       <c r="C21" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Pix2Graph</t>
+          <t>Pix2Graph</t>
         </is>
       </c>
       <c r="D21" s="84" t="inlineStr">
@@ -3573,35 +3590,35 @@
           <t>Inference-only (khong train); Qwen2.5-VL-3B sinh graph + tra loi VQA</t>
         </is>
       </c>
-      <c r="G21" s="84" t="n">
+      <c r="G21" s="137" t="n">
         <v>0.485</v>
       </c>
-      <c r="H21" s="84" t="n">
+      <c r="H21" s="137" t="n">
         <v>0.4463</v>
       </c>
-      <c r="I21" s="84" t="n">
+      <c r="I21" s="137" t="n">
         <v>0.448</v>
       </c>
-      <c r="J21" s="84" t="n">
+      <c r="J21" s="137" t="n">
         <v>0.4327</v>
       </c>
-      <c r="K21" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L21" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M21" s="84" t="n">
+      <c r="K21" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L21" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M21" s="137" t="n">
         <v>0.0014</v>
       </c>
-      <c r="N21" s="84" t="n">
+      <c r="N21" s="137" t="n">
         <v>0.552</v>
       </c>
-      <c r="O21" s="84" t="n">
+      <c r="O21" s="138" t="n">
         <v>1575.4</v>
       </c>
       <c r="P21" s="84" t="inlineStr">
@@ -3614,7 +3631,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R21" s="91" t="n">
+      <c r="R21" s="141" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="24" t="inlineStr">
@@ -3630,7 +3647,7 @@
       </c>
       <c r="C22" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">       MR-MKG</t>
+          <t>MR-MKG</t>
         </is>
       </c>
       <c r="D22" s="84" t="inlineStr">
@@ -3648,35 +3665,35 @@
           <t>Inference-only (khong train); Qwen2.5-VL-3B lam VLM + MMKG builder</t>
         </is>
       </c>
-      <c r="G22" s="84" t="n">
+      <c r="G22" s="137" t="n">
         <v>0.46</v>
       </c>
-      <c r="H22" s="84" t="n">
+      <c r="H22" s="137" t="n">
         <v>0.4227</v>
       </c>
-      <c r="I22" s="84" t="n">
+      <c r="I22" s="137" t="n">
         <v>0.4112</v>
       </c>
-      <c r="J22" s="84" t="n">
+      <c r="J22" s="137" t="n">
         <v>0.4005</v>
       </c>
-      <c r="K22" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L22" s="84" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M22" s="84" t="n">
+      <c r="K22" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L22" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M22" s="137" t="n">
         <v>0.0014</v>
       </c>
-      <c r="N22" s="84" t="n">
+      <c r="N22" s="137" t="n">
         <v>0.5888</v>
       </c>
-      <c r="O22" s="84" t="n">
+      <c r="O22" s="138" t="n">
         <v>1945.4</v>
       </c>
       <c r="P22" s="84" t="inlineStr">
@@ -3689,7 +3706,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="R22" s="84" t="n">
+      <c r="R22" s="139" t="n">
         <v>0</v>
       </c>
       <c r="S22" s="24" t="inlineStr">
@@ -3711,18 +3728,18 @@
       <c r="D23" s="96" t="n"/>
       <c r="E23" s="96" t="n"/>
       <c r="F23" s="96" t="n"/>
-      <c r="G23" s="84" t="n"/>
-      <c r="H23" s="84" t="n"/>
-      <c r="I23" s="84" t="n"/>
-      <c r="J23" s="84" t="n"/>
-      <c r="K23" s="84" t="n"/>
-      <c r="L23" s="84" t="n"/>
-      <c r="M23" s="84" t="n"/>
-      <c r="N23" s="84" t="n"/>
-      <c r="O23" s="84" t="n"/>
+      <c r="G23" s="137" t="n"/>
+      <c r="H23" s="137" t="n"/>
+      <c r="I23" s="137" t="n"/>
+      <c r="J23" s="137" t="n"/>
+      <c r="K23" s="137" t="n"/>
+      <c r="L23" s="137" t="n"/>
+      <c r="M23" s="137" t="n"/>
+      <c r="N23" s="137" t="n"/>
+      <c r="O23" s="138" t="n"/>
       <c r="P23" s="84" t="n"/>
       <c r="Q23" s="84" t="n"/>
-      <c r="R23" s="84" t="n"/>
+      <c r="R23" s="139" t="n"/>
       <c r="S23" s="100" t="n"/>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Fill #15 LLM4SGG real metrics (n=200) into Implement r23
Acc 0.455, P/R/F1 0.4628/0.4566/0.4444, FPR/FNR 0.001/0.5434, TrainTime
2664.1s, Steps 0 (inference-only). Graph-injected 0.455 vs baseline 0.46
(gain -0.005): the weakly-supervised caption-graph adds little over direct
VQA on these questions -- honest adaptation result, logged in Note.
Completes all 5 papers (#11-#15) in the sheet.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JOUR-2026.xlsx
+++ b/JOUR-2026.xlsx
@@ -3725,22 +3725,70 @@
           <t>LLM4SGG</t>
         </is>
       </c>
-      <c r="D23" s="96" t="n"/>
-      <c r="E23" s="96" t="n"/>
-      <c r="F23" s="96" t="n"/>
-      <c r="G23" s="137" t="n"/>
-      <c r="H23" s="137" t="n"/>
-      <c r="I23" s="137" t="n"/>
-      <c r="J23" s="137" t="n"/>
-      <c r="K23" s="137" t="n"/>
-      <c r="L23" s="137" t="n"/>
-      <c r="M23" s="137" t="n"/>
-      <c r="N23" s="137" t="n"/>
-      <c r="O23" s="138" t="n"/>
-      <c r="P23" s="84" t="n"/>
-      <c r="Q23" s="84" t="n"/>
-      <c r="R23" s="139" t="n"/>
-      <c r="S23" s="100" t="n"/>
+      <c r="D23" s="96" t="inlineStr">
+        <is>
+          <t>Weakly-supervised Scene Graph Generation -&gt; adapt sang graph-injected VQA</t>
+        </is>
+      </c>
+      <c r="E23" s="96" t="inlineStr">
+        <is>
+          <t>VLM caption -&gt; LLM CoT+few-shot triplet extraction (constrained predicate vocab) -&gt; scene graph -&gt; inject as VQA context</t>
+        </is>
+      </c>
+      <c r="F23" s="96" t="inlineStr">
+        <is>
+          <t>Inference-only (khong train); Qwen2.5-VL-3B lam VLM caption + LLM extractor</t>
+        </is>
+      </c>
+      <c r="G23" s="137" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="H23" s="137" t="n">
+        <v>0.4628</v>
+      </c>
+      <c r="I23" s="137" t="n">
+        <v>0.4566</v>
+      </c>
+      <c r="J23" s="137" t="n">
+        <v>0.4444</v>
+      </c>
+      <c r="K23" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L23" s="137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M23" s="137" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="N23" s="137" t="n">
+        <v>0.5434</v>
+      </c>
+      <c r="O23" s="138" t="n">
+        <v>2664.1</v>
+      </c>
+      <c r="P23" s="84" t="inlineStr">
+        <is>
+          <t>~3B (4bit=False); inference-only</t>
+        </is>
+      </c>
+      <c r="Q23" s="84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R23" s="139" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="100" t="inlineStr">
+        <is>
+          <t>Qwen2.5-VL-3B; Visual CoT-GQA; eval=200; inference-only (Steps=0). ADAPTATION: LLM4SGG goc = weakly-supervised SGG: dung CAPTION (text) thay vi dense bbox (weak supervision); LLM (GPT-3.5/4 trong paper) voi CoT + few-shot + predicate vocab trich (subject,predicate,object) tu caption -&gt; scene graph; benchmark VG/GQA, metric Recall@K. -&gt; Adapt (Huong A): VLM tu sinh caption (64 tok; KHONG dung gold reasoning/thought) -&gt; Qwen (che do text) CoT+2-few-shot+20-predicate-vocab trich triplets (align predicate ve vocab, giong class align cua paper) -&gt; scene graph (cap 10) -&gt; inject nhu VQA context -&gt; tra loi. Giu nguyen dong gop dac trung: text-mediated (caption-&gt;LLM), weak supervision, no bbox. Graph-inj Acc=0.4550; baseline Acc=0.4600 (gain -0.0050). Recall@K/ROC/PR-AUC=N/A (EM VQA, khong rerank). Faithful VG/GQA Recall@K + full predicate alignment + GPT-4 = future work. adaptation, not full LLM4SGG reproduction.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>

</xml_diff>